<commit_message>
Primera prueba realizada. Fallos cuando alcance diferente de mecanismo
</commit_message>
<xml_diff>
--- a/GeoMIP/results/Pruebas_iniciales_Metodo2.xlsx
+++ b/GeoMIP/results/Pruebas_iniciales_Metodo2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Universidad\ADA\proyecto\analisis-project-20261\GeoMIP\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C264DABA-493E-41C4-8860-4063894F53C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87FD23EB-2BAC-4F5D-8C64-4A68198D4D25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="plataformas" sheetId="1" r:id="rId1"/>
@@ -1259,16 +1259,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1505,9 +1505,9 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A2" s="8"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="10"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="13"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4"/>
@@ -2644,9 +2644,9 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18.140625" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.5703125" customWidth="1"/>
     <col min="6" max="6" width="22.42578125" customWidth="1"/>
     <col min="7" max="7" width="19.42578125" customWidth="1"/>
@@ -2704,11 +2704,11 @@
       <c r="AB1" s="5"/>
     </row>
     <row r="2" spans="1:28">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="13"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="10"/>
       <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
@@ -5714,11 +5714,11 @@
       <c r="AB1" s="5"/>
     </row>
     <row r="2" spans="1:28">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="13"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="10"/>
       <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
@@ -8758,11 +8758,11 @@
       <c r="AB1" s="5"/>
     </row>
     <row r="2" spans="1:28">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="13"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="10"/>
       <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
@@ -11802,11 +11802,11 @@
       <c r="AB1" s="5"/>
     </row>
     <row r="2" spans="1:28">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="13"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="10"/>
       <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
@@ -14990,11 +14990,11 @@
       <c r="AB1" s="5"/>
     </row>
     <row r="2" spans="1:28">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="13"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="10"/>
       <c r="D2" s="1" t="s">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
Optimización hecha. Aún no funciona para N=25
</commit_message>
<xml_diff>
--- a/GeoMIP/results/Pruebas_iniciales_Metodo2.xlsx
+++ b/GeoMIP/results/Pruebas_iniciales_Metodo2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Universidad\ADA\proyecto\analisis-project-20261\GeoMIP\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87FD23EB-2BAC-4F5D-8C64-4A68198D4D25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449FF5B2-DED9-4EA8-B77F-A1E74A6C96BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="plataformas" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="350">
   <si>
     <t>Unnamed: 0</t>
   </si>
@@ -903,9 +903,6 @@
   </si>
   <si>
     <t>Sistema Candidato: ABCDEFGHIJKLMNOPQRSTUVWXY</t>
-  </si>
-  <si>
-    <t>1000000000000000000000000</t>
   </si>
   <si>
     <t>ABCDEFGHIJKLMNOPQRSTUVWXY_{t+1}|ABCDEFGHIJKLMNOPQRSTUVWXY_{t}</t>
@@ -1238,7 +1235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1269,6 +1266,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14933,7 +14933,7 @@
     <col min="2" max="2" width="81.28515625" customWidth="1"/>
     <col min="3" max="3" width="29.28515625" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="25.5703125" customWidth="1"/>
+    <col min="5" max="5" width="29.140625" customWidth="1"/>
     <col min="6" max="6" width="22.42578125" customWidth="1"/>
     <col min="7" max="7" width="19.42578125" customWidth="1"/>
     <col min="8" max="8" width="19.28515625" customWidth="1"/>
@@ -14998,8 +14998,8 @@
       <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>285</v>
+      <c r="E2" s="14">
+        <v>9.9999999999999998E+23</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
@@ -15118,13 +15118,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>287</v>
-      </c>
       <c r="D4" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
@@ -15156,13 +15156,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>288</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>289</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
@@ -15194,13 +15194,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>290</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>291</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
@@ -15232,13 +15232,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>292</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>293</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
@@ -15270,13 +15270,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>294</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>295</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
@@ -15308,13 +15308,13 @@
         <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>296</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>297</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
@@ -15346,13 +15346,13 @@
         <v>7</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>298</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>299</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
@@ -15384,13 +15384,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
@@ -15422,13 +15422,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
@@ -15460,13 +15460,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
@@ -15498,13 +15498,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
@@ -15536,13 +15536,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
@@ -15574,13 +15574,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
@@ -15612,13 +15612,13 @@
         <v>14</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
@@ -15650,13 +15650,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
@@ -15688,13 +15688,13 @@
         <v>16</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
@@ -15726,13 +15726,13 @@
         <v>17</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
@@ -15764,13 +15764,13 @@
         <v>18</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
@@ -15802,13 +15802,13 @@
         <v>19</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
@@ -15840,13 +15840,13 @@
         <v>20</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
@@ -15878,13 +15878,13 @@
         <v>21</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
@@ -15916,13 +15916,13 @@
         <v>22</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
@@ -15954,13 +15954,13 @@
         <v>23</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
@@ -15992,13 +15992,13 @@
         <v>24</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
@@ -16030,13 +16030,13 @@
         <v>25</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
@@ -16068,13 +16068,13 @@
         <v>26</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
@@ -16106,13 +16106,13 @@
         <v>27</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
@@ -16144,13 +16144,13 @@
         <v>28</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
@@ -16182,13 +16182,13 @@
         <v>29</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
@@ -16220,13 +16220,13 @@
         <v>30</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
@@ -16258,13 +16258,13 @@
         <v>31</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
@@ -16296,13 +16296,13 @@
         <v>32</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
@@ -16334,13 +16334,13 @@
         <v>33</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
@@ -16372,13 +16372,13 @@
         <v>34</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
@@ -16410,13 +16410,13 @@
         <v>35</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
@@ -16448,13 +16448,13 @@
         <v>36</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
@@ -16486,13 +16486,13 @@
         <v>37</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
@@ -16524,13 +16524,13 @@
         <v>38</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
@@ -16562,13 +16562,13 @@
         <v>39</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
@@ -16600,13 +16600,13 @@
         <v>40</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
@@ -16638,13 +16638,13 @@
         <v>41</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
@@ -16676,13 +16676,13 @@
         <v>42</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
@@ -16714,13 +16714,13 @@
         <v>43</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
@@ -16752,13 +16752,13 @@
         <v>44</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
@@ -16790,13 +16790,13 @@
         <v>45</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
@@ -16828,13 +16828,13 @@
         <v>46</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
@@ -16866,13 +16866,13 @@
         <v>47</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
@@ -16904,13 +16904,13 @@
         <v>48</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
@@ -16942,13 +16942,13 @@
         <v>49</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E52" s="4"/>
       <c r="F52" s="4"/>
@@ -16980,13 +16980,13 @@
         <v>50</v>
       </c>
       <c r="B53" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="C53" s="4" t="s">
         <v>342</v>
       </c>
-      <c r="C53" s="4" t="s">
-        <v>343</v>
-      </c>
       <c r="D53" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
@@ -17979,37 +17979,37 @@
   <sheetData>
     <row r="1" spans="1:1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="14.25" customHeight="1">
       <c r="A2" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="4" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="4" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="4" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="4" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>